<commit_message>
Update wheat trait ontology add unspecified race stem rust infection trait
</commit_message>
<xml_diff>
--- a/ontology/triticum-props.xlsx
+++ b/ontology/triticum-props.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="923" uniqueCount="586">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="927" uniqueCount="588">
   <si>
     <t>trait_name</t>
   </si>
@@ -1772,6 +1772,12 @@
   </si>
   <si>
     <t>TRAIT: Agronomic appearance ::: METHOD: Agronomic Appearance Visual Estimation ::: SCALE: 0-9 Agronomic Appearance Scale</t>
+  </si>
+  <si>
+    <t>Stem rust seedling infection type - 0-9 Linearized Stakman Scale Rating</t>
+  </si>
+  <si>
+    <t>TRAIT: Stem rust seedling infection type ::: METHOD: Rust Infection Type Estimation ::: SCALE: 0-9 Linearized Stakman Scale Rating</t>
   </si>
 </sst>
 </file>
@@ -2103,7 +2109,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H278"/>
+  <dimension ref="A1:H279"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
@@ -6529,6 +6535,26 @@
         <v>585</v>
       </c>
     </row>
+    <row r="279" spans="1:7">
+      <c r="A279" t="s">
+        <v>586</v>
+      </c>
+      <c r="B279" t="s">
+        <v>13</v>
+      </c>
+      <c r="D279">
+        <v>0</v>
+      </c>
+      <c r="E279">
+        <v>9</v>
+      </c>
+      <c r="F279" t="s">
+        <v>16</v>
+      </c>
+      <c r="G279" t="s">
+        <v>587</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Update wheat trait ontology - add hessian fly rating traits
</commit_message>
<xml_diff>
--- a/ontology/triticum-props.xlsx
+++ b/ontology/triticum-props.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="927" uniqueCount="588">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="966" uniqueCount="612">
   <si>
     <t>trait_name</t>
   </si>
@@ -1778,6 +1778,78 @@
   </si>
   <si>
     <t>TRAIT: Stem rust seedling infection type ::: METHOD: Rust Infection Type Estimation ::: SCALE: 0-9 Linearized Stakman Scale Rating</t>
+  </si>
+  <si>
+    <t>Hessian fly rating - R</t>
+  </si>
+  <si>
+    <t>TRAIT: Hessian fly rating ::: METHOD: Hessian Fly Rating - Resistant Count ::: SCALE: plant/plot</t>
+  </si>
+  <si>
+    <t>Hessian fly rating - S</t>
+  </si>
+  <si>
+    <t>TRAIT: Hessian fly rating ::: METHOD: Hessian Fly Rating - Susceptible Count ::: SCALE: plant/plot</t>
+  </si>
+  <si>
+    <t>Hessian fly rating - %</t>
+  </si>
+  <si>
+    <t>TRAIT: Hessian fly rating ::: METHOD: Hessian Fly Rating - Resistant Percentage ::: SCALE: %</t>
+  </si>
+  <si>
+    <t>Hessian fly rating - GP - R</t>
+  </si>
+  <si>
+    <t>TRAIT: Hessian fly rating ::: METHOD: Hessian Fly Rating - GP - Resistant Count ::: SCALE: plant/plot</t>
+  </si>
+  <si>
+    <t>Hessian fly rating - GP - S</t>
+  </si>
+  <si>
+    <t>TRAIT: Hessian fly rating ::: METHOD: Hessian Fly Rating - GP - Susceptible Count ::: SCALE: plant/plot</t>
+  </si>
+  <si>
+    <t>Hessian fly rating - GP - %</t>
+  </si>
+  <si>
+    <t>TRAIT: Hessian fly rating ::: METHOD: Hessian Fly Rating - GP - Resistant Percentage ::: SCALE: %</t>
+  </si>
+  <si>
+    <t>Hessian fly rating - TX - R</t>
+  </si>
+  <si>
+    <t>TRAIT: Hessian fly rating ::: METHOD: Hessian Fly Rating - TX - Resistant Count ::: SCALE: plant/plot</t>
+  </si>
+  <si>
+    <t>Hessian fly rating - TX - S</t>
+  </si>
+  <si>
+    <t>TRAIT: Hessian fly rating ::: METHOD: Hessian Fly Rating - TX - Susceptible Count ::: SCALE: plant/plot</t>
+  </si>
+  <si>
+    <t>Hessian fly rating - TX - %</t>
+  </si>
+  <si>
+    <t>TRAIT: Hessian fly rating ::: METHOD: Hessian Fly Rating - TX - Resistant Percentage ::: SCALE: %</t>
+  </si>
+  <si>
+    <t>Hessian fly rating - 1-4 Rating Scale</t>
+  </si>
+  <si>
+    <t>TRAIT: Hessian fly rating ::: METHOD: Hessian Fly Rating - 1 to 4 Resistance Scale Estimation ::: SCALE: 1-4 HF resistance scale</t>
+  </si>
+  <si>
+    <t>Hessian fly rating - GP - 1-4 Rating Scale</t>
+  </si>
+  <si>
+    <t>TRAIT: Hessian fly rating ::: METHOD: Hessian Fly Rating - GP - 1 to 4 Resistance Scale Estimation ::: SCALE: 1-4 HF resistance scale</t>
+  </si>
+  <si>
+    <t>Hessian fly rating - TX - 1-4 Rating Scale</t>
+  </si>
+  <si>
+    <t>TRAIT: Hessian fly rating ::: METHOD: Hessian Fly Rating - TX - 1 to 4 Resistance Scale Estimation ::: SCALE: 1-4 HF resistance scale</t>
   </si>
 </sst>
 </file>
@@ -2109,7 +2181,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H279"/>
+  <dimension ref="A1:H291"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
@@ -6555,6 +6627,183 @@
         <v>587</v>
       </c>
     </row>
+    <row r="280" spans="1:7">
+      <c r="A280" t="s">
+        <v>588</v>
+      </c>
+      <c r="B280" t="s">
+        <v>13</v>
+      </c>
+      <c r="G280" t="s">
+        <v>589</v>
+      </c>
+    </row>
+    <row r="281" spans="1:7">
+      <c r="A281" t="s">
+        <v>590</v>
+      </c>
+      <c r="B281" t="s">
+        <v>13</v>
+      </c>
+      <c r="G281" t="s">
+        <v>591</v>
+      </c>
+    </row>
+    <row r="282" spans="1:7">
+      <c r="A282" t="s">
+        <v>592</v>
+      </c>
+      <c r="B282" t="s">
+        <v>13</v>
+      </c>
+      <c r="D282">
+        <v>0</v>
+      </c>
+      <c r="E282">
+        <v>100</v>
+      </c>
+      <c r="G282" t="s">
+        <v>593</v>
+      </c>
+    </row>
+    <row r="283" spans="1:7">
+      <c r="A283" t="s">
+        <v>594</v>
+      </c>
+      <c r="B283" t="s">
+        <v>13</v>
+      </c>
+      <c r="G283" t="s">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="284" spans="1:7">
+      <c r="A284" t="s">
+        <v>596</v>
+      </c>
+      <c r="B284" t="s">
+        <v>13</v>
+      </c>
+      <c r="G284" t="s">
+        <v>597</v>
+      </c>
+    </row>
+    <row r="285" spans="1:7">
+      <c r="A285" t="s">
+        <v>598</v>
+      </c>
+      <c r="B285" t="s">
+        <v>13</v>
+      </c>
+      <c r="D285">
+        <v>0</v>
+      </c>
+      <c r="E285">
+        <v>100</v>
+      </c>
+      <c r="G285" t="s">
+        <v>599</v>
+      </c>
+    </row>
+    <row r="286" spans="1:7">
+      <c r="A286" t="s">
+        <v>600</v>
+      </c>
+      <c r="B286" t="s">
+        <v>13</v>
+      </c>
+      <c r="G286" t="s">
+        <v>601</v>
+      </c>
+    </row>
+    <row r="287" spans="1:7">
+      <c r="A287" t="s">
+        <v>602</v>
+      </c>
+      <c r="B287" t="s">
+        <v>13</v>
+      </c>
+      <c r="G287" t="s">
+        <v>603</v>
+      </c>
+    </row>
+    <row r="288" spans="1:7">
+      <c r="A288" t="s">
+        <v>604</v>
+      </c>
+      <c r="B288" t="s">
+        <v>13</v>
+      </c>
+      <c r="D288">
+        <v>0</v>
+      </c>
+      <c r="E288">
+        <v>100</v>
+      </c>
+      <c r="G288" t="s">
+        <v>605</v>
+      </c>
+    </row>
+    <row r="289" spans="1:7">
+      <c r="A289" t="s">
+        <v>606</v>
+      </c>
+      <c r="B289" t="s">
+        <v>9</v>
+      </c>
+      <c r="D289">
+        <v>1</v>
+      </c>
+      <c r="E289">
+        <v>4</v>
+      </c>
+      <c r="F289" t="s">
+        <v>268</v>
+      </c>
+      <c r="G289" t="s">
+        <v>607</v>
+      </c>
+    </row>
+    <row r="290" spans="1:7">
+      <c r="A290" t="s">
+        <v>608</v>
+      </c>
+      <c r="B290" t="s">
+        <v>9</v>
+      </c>
+      <c r="D290">
+        <v>1</v>
+      </c>
+      <c r="E290">
+        <v>4</v>
+      </c>
+      <c r="F290" t="s">
+        <v>268</v>
+      </c>
+      <c r="G290" t="s">
+        <v>609</v>
+      </c>
+    </row>
+    <row r="291" spans="1:7">
+      <c r="A291" t="s">
+        <v>610</v>
+      </c>
+      <c r="B291" t="s">
+        <v>9</v>
+      </c>
+      <c r="D291">
+        <v>1</v>
+      </c>
+      <c r="E291">
+        <v>4</v>
+      </c>
+      <c r="F291" t="s">
+        <v>268</v>
+      </c>
+      <c r="G291" t="s">
+        <v>611</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Update wheat trait ontology improve hessian fly resistance trait names
</commit_message>
<xml_diff>
--- a/ontology/triticum-props.xlsx
+++ b/ontology/triticum-props.xlsx
@@ -1780,76 +1780,76 @@
     <t>TRAIT: Stem rust seedling infection type ::: METHOD: Rust Infection Type Estimation ::: SCALE: 0-9 Linearized Stakman Scale Rating</t>
   </si>
   <si>
-    <t>Hessian fly rating - R</t>
-  </si>
-  <si>
-    <t>TRAIT: Hessian fly rating ::: METHOD: Hessian Fly Rating - Resistant Count ::: SCALE: plant/plot</t>
-  </si>
-  <si>
-    <t>Hessian fly rating - S</t>
-  </si>
-  <si>
-    <t>TRAIT: Hessian fly rating ::: METHOD: Hessian Fly Rating - Susceptible Count ::: SCALE: plant/plot</t>
-  </si>
-  <si>
-    <t>Hessian fly rating - %</t>
-  </si>
-  <si>
-    <t>TRAIT: Hessian fly rating ::: METHOD: Hessian Fly Rating - Resistant Percentage ::: SCALE: %</t>
-  </si>
-  <si>
-    <t>Hessian fly rating - GP - R</t>
-  </si>
-  <si>
-    <t>TRAIT: Hessian fly rating ::: METHOD: Hessian Fly Rating - GP - Resistant Count ::: SCALE: plant/plot</t>
-  </si>
-  <si>
-    <t>Hessian fly rating - GP - S</t>
-  </si>
-  <si>
-    <t>TRAIT: Hessian fly rating ::: METHOD: Hessian Fly Rating - GP - Susceptible Count ::: SCALE: plant/plot</t>
-  </si>
-  <si>
-    <t>Hessian fly rating - GP - %</t>
-  </si>
-  <si>
-    <t>TRAIT: Hessian fly rating ::: METHOD: Hessian Fly Rating - GP - Resistant Percentage ::: SCALE: %</t>
-  </si>
-  <si>
-    <t>Hessian fly rating - TX - R</t>
-  </si>
-  <si>
-    <t>TRAIT: Hessian fly rating ::: METHOD: Hessian Fly Rating - TX - Resistant Count ::: SCALE: plant/plot</t>
-  </si>
-  <si>
-    <t>Hessian fly rating - TX - S</t>
-  </si>
-  <si>
-    <t>TRAIT: Hessian fly rating ::: METHOD: Hessian Fly Rating - TX - Susceptible Count ::: SCALE: plant/plot</t>
-  </si>
-  <si>
-    <t>Hessian fly rating - TX - %</t>
-  </si>
-  <si>
-    <t>TRAIT: Hessian fly rating ::: METHOD: Hessian Fly Rating - TX - Resistant Percentage ::: SCALE: %</t>
-  </si>
-  <si>
-    <t>Hessian fly rating - 1-4 Rating Scale</t>
-  </si>
-  <si>
-    <t>TRAIT: Hessian fly rating ::: METHOD: Hessian Fly Rating - 1 to 4 Resistance Scale Estimation ::: SCALE: 1-4 HF resistance scale</t>
-  </si>
-  <si>
-    <t>Hessian fly rating - GP - 1-4 Rating Scale</t>
-  </si>
-  <si>
-    <t>TRAIT: Hessian fly rating ::: METHOD: Hessian Fly Rating - GP - 1 to 4 Resistance Scale Estimation ::: SCALE: 1-4 HF resistance scale</t>
-  </si>
-  <si>
-    <t>Hessian fly rating - TX - 1-4 Rating Scale</t>
-  </si>
-  <si>
-    <t>TRAIT: Hessian fly rating ::: METHOD: Hessian Fly Rating - TX - 1 to 4 Resistance Scale Estimation ::: SCALE: 1-4 HF resistance scale</t>
+    <t>Hessian fly resistance rating - R</t>
+  </si>
+  <si>
+    <t>TRAIT: Hessian fly resistance rating ::: METHOD: Hessian Fly Rating - Resistant Count ::: SCALE: plant/plot</t>
+  </si>
+  <si>
+    <t>Hessian fly resistance rating - S</t>
+  </si>
+  <si>
+    <t>TRAIT: Hessian fly resistance rating ::: METHOD: Hessian Fly Rating - Susceptible Count ::: SCALE: plant/plot</t>
+  </si>
+  <si>
+    <t>Hessian fly resistance rating - %R</t>
+  </si>
+  <si>
+    <t>TRAIT: Hessian fly resistance rating ::: METHOD: Hessian Fly Rating - Resistant Percentage ::: SCALE: %</t>
+  </si>
+  <si>
+    <t>Hessian fly resistance rating - GP - R</t>
+  </si>
+  <si>
+    <t>TRAIT: Hessian fly resistance rating ::: METHOD: Hessian Fly Rating - GP - Resistant Count ::: SCALE: plant/plot</t>
+  </si>
+  <si>
+    <t>Hessian fly resistance rating - GP - S</t>
+  </si>
+  <si>
+    <t>TRAIT: Hessian fly resistance rating ::: METHOD: Hessian Fly Rating - GP - Susceptible Count ::: SCALE: plant/plot</t>
+  </si>
+  <si>
+    <t>Hessian fly resistance rating - GP - %R</t>
+  </si>
+  <si>
+    <t>TRAIT: Hessian fly resistance rating ::: METHOD: Hessian Fly Rating - GP - Resistant Percentage ::: SCALE: %</t>
+  </si>
+  <si>
+    <t>Hessian fly resistance rating - TX - R</t>
+  </si>
+  <si>
+    <t>TRAIT: Hessian fly resistance rating ::: METHOD: Hessian Fly Rating - TX - Resistant Count ::: SCALE: plant/plot</t>
+  </si>
+  <si>
+    <t>Hessian fly resistance rating - TX - S</t>
+  </si>
+  <si>
+    <t>TRAIT: Hessian fly resistance rating ::: METHOD: Hessian Fly Rating - TX - Susceptible Count ::: SCALE: plant/plot</t>
+  </si>
+  <si>
+    <t>Hessian fly resistance rating - TX - %R</t>
+  </si>
+  <si>
+    <t>TRAIT: Hessian fly resistance rating ::: METHOD: Hessian Fly Rating - TX - Resistant Percentage ::: SCALE: %</t>
+  </si>
+  <si>
+    <t>Hessian fly resistance rating - 1-4 Rating Scale</t>
+  </si>
+  <si>
+    <t>TRAIT: Hessian fly resistance rating ::: METHOD: Hessian Fly Rating - 1 to 4 Resistance Scale Estimation ::: SCALE: 1-4 HF resistance scale</t>
+  </si>
+  <si>
+    <t>Hessian fly resistance rating - GP - 1-4 Rating Scale</t>
+  </si>
+  <si>
+    <t>TRAIT: Hessian fly resistance rating ::: METHOD: Hessian Fly Rating - GP - 1 to 4 Resistance Scale Estimation ::: SCALE: 1-4 HF resistance scale</t>
+  </si>
+  <si>
+    <t>Hessian fly resistance rating - TX - 1-4 Rating Scale</t>
+  </si>
+  <si>
+    <t>TRAIT: Hessian fly resistance rating ::: METHOD: Hessian Fly Rating - TX - 1 to 4 Resistance Scale Estimation ::: SCALE: 1-4 HF resistance scale</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Wheat Traits: add green leaf area - % trait
</commit_message>
<xml_diff>
--- a/ontology/triticum-props.xlsx
+++ b/ontology/triticum-props.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="966" uniqueCount="612">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="969" uniqueCount="614">
   <si>
     <t>trait_name</t>
   </si>
@@ -1850,6 +1850,12 @@
   </si>
   <si>
     <t>TRAIT: Hessian fly resistance rating ::: METHOD: Hessian Fly Rating - TX - 1 to 4 Resistance Scale Estimation ::: SCALE: 1-4 HF resistance scale</t>
+  </si>
+  <si>
+    <t>Green leaf area - %</t>
+  </si>
+  <si>
+    <t>TRAIT: Green leaf area ::: METHOD: Green Leaf Area Estimation ::: SCALE: %</t>
   </si>
 </sst>
 </file>
@@ -2181,7 +2187,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H291"/>
+  <dimension ref="A1:H292"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
@@ -6804,6 +6810,23 @@
         <v>611</v>
       </c>
     </row>
+    <row r="292" spans="1:7">
+      <c r="A292" t="s">
+        <v>612</v>
+      </c>
+      <c r="B292" t="s">
+        <v>13</v>
+      </c>
+      <c r="D292">
+        <v>0</v>
+      </c>
+      <c r="E292">
+        <v>100</v>
+      </c>
+      <c r="G292" t="s">
+        <v>613</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Wheat Ontology: add grain purple proportion trait
</commit_message>
<xml_diff>
--- a/ontology/triticum-props.xlsx
+++ b/ontology/triticum-props.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="969" uniqueCount="614">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="963" uniqueCount="616">
   <si>
     <t>trait_name</t>
   </si>
@@ -1856,6 +1856,12 @@
   </si>
   <si>
     <t>TRAIT: Green leaf area ::: METHOD: Green Leaf Area Estimation ::: SCALE: %</t>
+  </si>
+  <si>
+    <t>Grain purple proportion - %</t>
+  </si>
+  <si>
+    <t>TRAIT: Grain purple proportion ::: METHOD: Grain Purple Proportion Estimation ::: SCALE: Grain purple proportion</t>
   </si>
 </sst>
 </file>
@@ -2187,7 +2193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H292"/>
+  <dimension ref="A1:H293"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
@@ -5058,9 +5064,6 @@
       <c r="E176">
         <v>9</v>
       </c>
-      <c r="F176" t="s">
-        <v>16</v>
-      </c>
       <c r="G176" t="s">
         <v>374</v>
       </c>
@@ -5078,9 +5081,6 @@
       <c r="E177">
         <v>9</v>
       </c>
-      <c r="F177" t="s">
-        <v>16</v>
-      </c>
       <c r="G177" t="s">
         <v>376</v>
       </c>
@@ -5098,9 +5098,6 @@
       <c r="E178">
         <v>9</v>
       </c>
-      <c r="F178" t="s">
-        <v>16</v>
-      </c>
       <c r="G178" t="s">
         <v>378</v>
       </c>
@@ -5118,9 +5115,6 @@
       <c r="E179">
         <v>9</v>
       </c>
-      <c r="F179" t="s">
-        <v>16</v>
-      </c>
       <c r="G179" t="s">
         <v>380</v>
       </c>
@@ -5138,9 +5132,6 @@
       <c r="E180">
         <v>9</v>
       </c>
-      <c r="F180" t="s">
-        <v>16</v>
-      </c>
       <c r="G180" t="s">
         <v>382</v>
       </c>
@@ -5158,9 +5149,6 @@
       <c r="E181">
         <v>9</v>
       </c>
-      <c r="F181" t="s">
-        <v>16</v>
-      </c>
       <c r="G181" t="s">
         <v>384</v>
       </c>
@@ -5516,9 +5504,6 @@
       <c r="E204">
         <v>9</v>
       </c>
-      <c r="F204" t="s">
-        <v>16</v>
-      </c>
       <c r="G204" t="s">
         <v>432</v>
       </c>
@@ -6422,9 +6407,6 @@
       <c r="E267">
         <v>5</v>
       </c>
-      <c r="F267" t="s">
-        <v>10</v>
-      </c>
       <c r="G267" t="s">
         <v>562</v>
       </c>
@@ -6626,9 +6608,6 @@
       <c r="E279">
         <v>9</v>
       </c>
-      <c r="F279" t="s">
-        <v>16</v>
-      </c>
       <c r="G279" t="s">
         <v>587</v>
       </c>
@@ -6825,6 +6804,23 @@
       </c>
       <c r="G292" t="s">
         <v>613</v>
+      </c>
+    </row>
+    <row r="293" spans="1:7">
+      <c r="A293" t="s">
+        <v>614</v>
+      </c>
+      <c r="B293" t="s">
+        <v>13</v>
+      </c>
+      <c r="D293">
+        <v>0</v>
+      </c>
+      <c r="E293">
+        <v>100</v>
+      </c>
+      <c r="G293" t="s">
+        <v>615</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update Wheat ontology add sawfly infestation trait
</commit_message>
<xml_diff>
--- a/ontology/triticum-props.xlsx
+++ b/ontology/triticum-props.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="963" uniqueCount="616">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="966" uniqueCount="618">
   <si>
     <t>trait_name</t>
   </si>
@@ -1862,6 +1862,12 @@
   </si>
   <si>
     <t>TRAIT: Grain purple proportion ::: METHOD: Grain Purple Proportion Estimation ::: SCALE: Grain purple proportion</t>
+  </si>
+  <si>
+    <t>Sawfly infestation - %</t>
+  </si>
+  <si>
+    <t>TRAIT: Sawfly infestation ::: METHOD: Sawfly Infestation Estimation ::: SCALE: %</t>
   </si>
 </sst>
 </file>
@@ -2193,7 +2199,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H293"/>
+  <dimension ref="A1:H294"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
@@ -6823,6 +6829,23 @@
         <v>615</v>
       </c>
     </row>
+    <row r="294" spans="1:7">
+      <c r="A294" t="s">
+        <v>616</v>
+      </c>
+      <c r="B294" t="s">
+        <v>13</v>
+      </c>
+      <c r="D294">
+        <v>0</v>
+      </c>
+      <c r="E294">
+        <v>100</v>
+      </c>
+      <c r="G294" t="s">
+        <v>617</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>